<commit_message>
Update checklist after second review
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#FONDAZIONEPADREALBERTOMILENOXX/Alessandro_DAlessandro/sgi-fse/2.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#FONDAZIONEPADREALBERTOMILENOXX/Alessandro_DAlessandro/sgi-fse/2.0/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alessandrodalessandro/pCloud sync/alex/Fondazione/Fondazione PHP/sgi/docs/FSE_ACCREDITAMENTO_SUBMISSION/GATEWAY/A1#111#FONDAZIONEPADREALBERTOMILENOXX/Alessandro_DAlessandro/sgi-fse/2.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFD8A6E0-8BEC-0446-B2F3-05A538A8DE73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4C4101-EE31-7B40-8671-8349A5030454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="920" yWindow="660" windowWidth="15740" windowHeight="14760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,6 +41,7 @@
             <sz val="11"/>
             <color theme="1"/>
             <rFont val="Calibri"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>======
@@ -55,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1744" uniqueCount="700">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1745" uniqueCount="700">
   <si>
     <t>NOME FORNITORE: Alessandro D'Alessandro</t>
   </si>
@@ -1501,9 +1502,6 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.99.999.1.1.b5eb4a5fdbd67ac2506b34952bb0e02feaf8905c1dfe11270e110a6019c98b96.3db767617f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>est eseguito con risposta attesa 400 dal Gateway: type /msg/syntax, detail "ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{\"urn:hl7-org:v3\":languageCode}'. One of '{\"urn:hl7-org:v3\":confidentialityCode}' is expected.". Evidenza ricavata da fse_transazioni id 38 del 31/03/2026.</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT27_KO</t>
@@ -2431,6 +2429,9 @@
   </si>
   <si>
     <t>Validazione respinta dal Gateway FSE: il documento LDO contiene errori sintattici e non puo' essere validato.</t>
+  </si>
+  <si>
+    <t>Test eseguito con risposta attesa 400 dal Gateway: type /msg/syntax, detail "ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{\"urn:hl7-org:v3\":languageCode}'. One of '{\"urn:hl7-org:v3\":confidentialityCode}' is expected.". Evidenza ricavata da fse_transazioni id 38 del 31/03/2026.</t>
   </si>
 </sst>
 </file>
@@ -3093,28 +3094,6 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3129,6 +3108,28 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3433,37 +3434,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="87" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="87" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="38" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="275.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="87" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
@@ -3471,17 +3472,17 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
@@ -3508,12 +3509,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="3" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="4" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -3524,7 +3525,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -3532,7 +3533,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -3540,7 +3541,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -3548,7 +3549,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
@@ -3556,7 +3557,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -3564,7 +3565,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4574,7 +4575,7 @@
     <col min="6" max="9" width="33.1640625" customWidth="1"/>
     <col min="10" max="10" width="27.1640625" customWidth="1"/>
     <col min="11" max="14" width="36.5" customWidth="1"/>
-    <col min="15" max="15" width="36.5" style="76" customWidth="1"/>
+    <col min="15" max="15" width="36.5" style="64" customWidth="1"/>
     <col min="16" max="18" width="36.5" customWidth="1"/>
     <col min="19" max="19" width="27.1640625" customWidth="1"/>
     <col min="20" max="20" width="33.1640625" customWidth="1"/>
@@ -4594,7 +4595,7 @@
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
       <c r="N1" s="7"/>
-      <c r="O1" s="72"/>
+      <c r="O1" s="60"/>
       <c r="P1" s="7"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="7"/>
@@ -4605,12 +4606,12 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="75" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="67"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="76"/>
+      <c r="D2" s="68"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -4620,7 +4621,7 @@
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
-      <c r="O2" s="72"/>
+      <c r="O2" s="60"/>
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
@@ -4631,14 +4632,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="60" t="s">
+      <c r="A3" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="61"/>
-      <c r="C3" s="69" t="s">
+      <c r="B3" s="70"/>
+      <c r="C3" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="67"/>
+      <c r="D3" s="68"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -4648,7 +4649,7 @@
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
-      <c r="O3" s="72"/>
+      <c r="O3" s="60"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
@@ -4659,12 +4660,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="62"/>
-      <c r="B4" s="63"/>
-      <c r="C4" s="69" t="s">
+      <c r="A4" s="71"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="67"/>
+      <c r="D4" s="68"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -4675,7 +4676,7 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
-      <c r="O4" s="72"/>
+      <c r="O4" s="60"/>
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
@@ -4686,12 +4687,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="64"/>
-      <c r="B5" s="65"/>
-      <c r="C5" s="69" t="s">
+      <c r="A5" s="73"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="67"/>
+      <c r="D5" s="68"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -4701,7 +4702,7 @@
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
-      <c r="O5" s="72"/>
+      <c r="O5" s="60"/>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
@@ -4712,8 +4713,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="70"/>
-      <c r="B6" s="71"/>
+      <c r="A6" s="65"/>
+      <c r="B6" s="66"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -4724,7 +4725,7 @@
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="7"/>
-      <c r="O6" s="72"/>
+      <c r="O6" s="60"/>
       <c r="P6" s="7"/>
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
@@ -4747,7 +4748,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
-      <c r="O7" s="72"/>
+      <c r="O7" s="60"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
@@ -4767,7 +4768,7 @@
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>
-      <c r="O8" s="72"/>
+      <c r="O8" s="60"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
@@ -4820,7 +4821,7 @@
       <c r="N9" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="O9" s="73" t="s">
+      <c r="O9" s="61" t="s">
         <v>19</v>
       </c>
       <c r="P9" s="17" t="s">
@@ -4961,8 +4962,8 @@
       <c r="N12" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O12" s="74" t="s">
-        <v>695</v>
+      <c r="O12" s="62" t="s">
+        <v>694</v>
       </c>
       <c r="P12" s="32" t="s">
         <v>42</v>
@@ -4974,7 +4975,7 @@
         <v>42</v>
       </c>
       <c r="S12" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T12" s="32" t="s">
         <v>43</v>
@@ -5287,8 +5288,8 @@
       <c r="N20" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O20" s="74" t="s">
-        <v>696</v>
+      <c r="O20" s="62" t="s">
+        <v>695</v>
       </c>
       <c r="P20" s="32" t="s">
         <v>42</v>
@@ -5300,7 +5301,7 @@
         <v>42</v>
       </c>
       <c r="S20" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T20" s="32" t="s">
         <v>43</v>
@@ -5607,7 +5608,7 @@
       <c r="N28" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O28" s="74" t="s">
+      <c r="O28" s="62" t="s">
         <v>72</v>
       </c>
       <c r="P28" s="32" t="s">
@@ -6202,8 +6203,8 @@
       <c r="N43" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O43" s="74" t="s">
-        <v>697</v>
+      <c r="O43" s="62" t="s">
+        <v>696</v>
       </c>
       <c r="P43" s="32" t="s">
         <v>42</v>
@@ -6215,7 +6216,7 @@
         <v>42</v>
       </c>
       <c r="S43" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T43" s="32" t="s">
         <v>43</v>
@@ -6269,8 +6270,8 @@
       <c r="N44" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O44" s="74" t="s">
-        <v>697</v>
+      <c r="O44" s="62" t="s">
+        <v>696</v>
       </c>
       <c r="P44" s="32" t="s">
         <v>42</v>
@@ -6282,7 +6283,7 @@
         <v>42</v>
       </c>
       <c r="S44" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T44" s="32" t="s">
         <v>43</v>
@@ -6336,8 +6337,8 @@
       <c r="N45" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O45" s="74" t="s">
-        <v>697</v>
+      <c r="O45" s="62" t="s">
+        <v>696</v>
       </c>
       <c r="P45" s="32" t="s">
         <v>42</v>
@@ -6349,7 +6350,7 @@
         <v>42</v>
       </c>
       <c r="S45" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T45" s="32" t="s">
         <v>43</v>
@@ -6403,8 +6404,8 @@
       <c r="N46" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O46" s="74" t="s">
-        <v>698</v>
+      <c r="O46" s="62" t="s">
+        <v>697</v>
       </c>
       <c r="P46" s="32" t="s">
         <v>42</v>
@@ -6416,7 +6417,7 @@
         <v>42</v>
       </c>
       <c r="S46" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T46" s="32" t="s">
         <v>43</v>
@@ -6470,8 +6471,8 @@
       <c r="N47" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O47" s="74" t="s">
-        <v>697</v>
+      <c r="O47" s="62" t="s">
+        <v>696</v>
       </c>
       <c r="P47" s="32" t="s">
         <v>42</v>
@@ -6483,7 +6484,7 @@
         <v>42</v>
       </c>
       <c r="S47" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T47" s="32" t="s">
         <v>43</v>
@@ -6537,8 +6538,8 @@
       <c r="N48" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O48" s="74" t="s">
-        <v>697</v>
+      <c r="O48" s="62" t="s">
+        <v>696</v>
       </c>
       <c r="P48" s="32" t="s">
         <v>42</v>
@@ -6550,7 +6551,7 @@
         <v>42</v>
       </c>
       <c r="S48" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T48" s="32" t="s">
         <v>43</v>
@@ -6604,8 +6605,8 @@
       <c r="N49" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O49" s="74" t="s">
-        <v>697</v>
+      <c r="O49" s="62" t="s">
+        <v>696</v>
       </c>
       <c r="P49" s="32" t="s">
         <v>42</v>
@@ -6617,7 +6618,7 @@
         <v>42</v>
       </c>
       <c r="S49" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T49" s="32" t="s">
         <v>43</v>
@@ -6671,8 +6672,8 @@
       <c r="N50" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O50" s="74" t="s">
-        <v>697</v>
+      <c r="O50" s="62" t="s">
+        <v>696</v>
       </c>
       <c r="P50" s="32" t="s">
         <v>42</v>
@@ -6684,7 +6685,7 @@
         <v>42</v>
       </c>
       <c r="S50" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T50" s="32" t="s">
         <v>43</v>
@@ -6738,8 +6739,8 @@
       <c r="N51" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O51" s="74" t="s">
-        <v>698</v>
+      <c r="O51" s="62" t="s">
+        <v>697</v>
       </c>
       <c r="P51" s="32" t="s">
         <v>42</v>
@@ -6751,7 +6752,7 @@
         <v>42</v>
       </c>
       <c r="S51" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T51" s="32" t="s">
         <v>43</v>
@@ -6805,7 +6806,9 @@
       <c r="N52" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O52" s="74"/>
+      <c r="O52" s="62" t="s">
+        <v>697</v>
+      </c>
       <c r="P52" s="32" t="s">
         <v>42</v>
       </c>
@@ -6816,7 +6819,7 @@
         <v>42</v>
       </c>
       <c r="S52" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T52" s="32" t="s">
         <v>43</v>
@@ -11049,8 +11052,8 @@
       <c r="L166" s="32"/>
       <c r="M166" s="32"/>
       <c r="N166" s="32"/>
-      <c r="O166" s="74" t="s">
-        <v>698</v>
+      <c r="O166" s="62" t="s">
+        <v>697</v>
       </c>
       <c r="P166" s="32"/>
       <c r="Q166" s="32"/>
@@ -11104,7 +11107,7 @@
       <c r="L167" s="32"/>
       <c r="M167" s="32"/>
       <c r="N167" s="32"/>
-      <c r="O167" s="74"/>
+      <c r="O167" s="62"/>
       <c r="P167" s="32"/>
       <c r="Q167" s="32"/>
       <c r="R167" s="32"/>
@@ -11679,8 +11682,8 @@
       <c r="N182" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="O182" s="75" t="s">
-        <v>699</v>
+      <c r="O182" s="63" t="s">
+        <v>698</v>
       </c>
       <c r="P182" s="32" t="s">
         <v>42</v>
@@ -11692,7 +11695,7 @@
         <v>42</v>
       </c>
       <c r="S182" s="32" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="T182" s="32" t="s">
         <v>43</v>
@@ -11701,7 +11704,7 @@
         <v>42</v>
       </c>
       <c r="V182" s="29" t="s">
-        <v>428</v>
+        <v>699</v>
       </c>
       <c r="W182" s="29" t="s">
         <v>35</v>
@@ -11718,10 +11721,10 @@
         <v>49</v>
       </c>
       <c r="D183" s="29" t="s">
+        <v>428</v>
+      </c>
+      <c r="E183" s="37" t="s">
         <v>429</v>
-      </c>
-      <c r="E183" s="37" t="s">
-        <v>430</v>
       </c>
       <c r="F183" s="29"/>
       <c r="G183" s="29"/>
@@ -11755,10 +11758,10 @@
         <v>45</v>
       </c>
       <c r="D184" s="29" t="s">
+        <v>430</v>
+      </c>
+      <c r="E184" s="37" t="s">
         <v>431</v>
-      </c>
-      <c r="E184" s="37" t="s">
-        <v>432</v>
       </c>
       <c r="F184" s="29"/>
       <c r="G184" s="29"/>
@@ -11792,10 +11795,10 @@
         <v>347</v>
       </c>
       <c r="D185" s="29" t="s">
+        <v>432</v>
+      </c>
+      <c r="E185" s="37" t="s">
         <v>433</v>
-      </c>
-      <c r="E185" s="37" t="s">
-        <v>434</v>
       </c>
       <c r="F185" s="29"/>
       <c r="G185" s="29"/>
@@ -11829,10 +11832,10 @@
         <v>47</v>
       </c>
       <c r="D186" s="29" t="s">
+        <v>434</v>
+      </c>
+      <c r="E186" s="37" t="s">
         <v>435</v>
-      </c>
-      <c r="E186" s="37" t="s">
-        <v>436</v>
       </c>
       <c r="F186" s="31"/>
       <c r="G186" s="31"/>
@@ -11866,10 +11869,10 @@
         <v>47</v>
       </c>
       <c r="D187" s="29" t="s">
+        <v>436</v>
+      </c>
+      <c r="E187" s="37" t="s">
         <v>437</v>
-      </c>
-      <c r="E187" s="37" t="s">
-        <v>438</v>
       </c>
       <c r="F187" s="31"/>
       <c r="G187" s="31"/>
@@ -11903,10 +11906,10 @@
         <v>29</v>
       </c>
       <c r="D188" s="35" t="s">
+        <v>438</v>
+      </c>
+      <c r="E188" s="37" t="s">
         <v>439</v>
-      </c>
-      <c r="E188" s="37" t="s">
-        <v>440</v>
       </c>
       <c r="F188" s="31"/>
       <c r="G188" s="31"/>
@@ -11940,10 +11943,10 @@
         <v>47</v>
       </c>
       <c r="D189" s="29" t="s">
+        <v>440</v>
+      </c>
+      <c r="E189" s="37" t="s">
         <v>441</v>
-      </c>
-      <c r="E189" s="37" t="s">
-        <v>442</v>
       </c>
       <c r="F189" s="31"/>
       <c r="G189" s="31"/>
@@ -11977,10 +11980,10 @@
         <v>49</v>
       </c>
       <c r="D190" s="29" t="s">
+        <v>442</v>
+      </c>
+      <c r="E190" s="37" t="s">
         <v>443</v>
-      </c>
-      <c r="E190" s="37" t="s">
-        <v>444</v>
       </c>
       <c r="F190" s="31"/>
       <c r="G190" s="31"/>
@@ -12014,10 +12017,10 @@
         <v>45</v>
       </c>
       <c r="D191" s="29" t="s">
+        <v>444</v>
+      </c>
+      <c r="E191" s="37" t="s">
         <v>445</v>
-      </c>
-      <c r="E191" s="37" t="s">
-        <v>446</v>
       </c>
       <c r="F191" s="31"/>
       <c r="G191" s="31"/>
@@ -12051,10 +12054,10 @@
         <v>45</v>
       </c>
       <c r="D192" s="29" t="s">
+        <v>446</v>
+      </c>
+      <c r="E192" s="37" t="s">
         <v>447</v>
-      </c>
-      <c r="E192" s="37" t="s">
-        <v>448</v>
       </c>
       <c r="F192" s="31"/>
       <c r="G192" s="31"/>
@@ -12088,10 +12091,10 @@
         <v>45</v>
       </c>
       <c r="D193" s="29" t="s">
+        <v>448</v>
+      </c>
+      <c r="E193" s="40" t="s">
         <v>449</v>
-      </c>
-      <c r="E193" s="40" t="s">
-        <v>450</v>
       </c>
       <c r="F193" s="31"/>
       <c r="G193" s="31"/>
@@ -12122,13 +12125,13 @@
         <v>28</v>
       </c>
       <c r="C194" s="35" t="s">
+        <v>450</v>
+      </c>
+      <c r="D194" s="29" t="s">
         <v>451</v>
       </c>
-      <c r="D194" s="29" t="s">
+      <c r="E194" s="40" t="s">
         <v>452</v>
-      </c>
-      <c r="E194" s="40" t="s">
-        <v>453</v>
       </c>
       <c r="F194" s="31"/>
       <c r="G194" s="31"/>
@@ -12159,13 +12162,13 @@
         <v>28</v>
       </c>
       <c r="C195" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D195" s="29" t="s">
+        <v>453</v>
+      </c>
+      <c r="E195" s="40" t="s">
         <v>454</v>
-      </c>
-      <c r="E195" s="40" t="s">
-        <v>455</v>
       </c>
       <c r="F195" s="31"/>
       <c r="G195" s="31"/>
@@ -12196,13 +12199,13 @@
         <v>28</v>
       </c>
       <c r="C196" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D196" s="29" t="s">
+        <v>455</v>
+      </c>
+      <c r="E196" s="40" t="s">
         <v>456</v>
-      </c>
-      <c r="E196" s="40" t="s">
-        <v>457</v>
       </c>
       <c r="F196" s="31"/>
       <c r="G196" s="31"/>
@@ -12233,13 +12236,13 @@
         <v>28</v>
       </c>
       <c r="C197" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D197" s="29" t="s">
+        <v>457</v>
+      </c>
+      <c r="E197" s="40" t="s">
         <v>458</v>
-      </c>
-      <c r="E197" s="40" t="s">
-        <v>459</v>
       </c>
       <c r="F197" s="31"/>
       <c r="G197" s="31"/>
@@ -12270,13 +12273,13 @@
         <v>28</v>
       </c>
       <c r="C198" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D198" s="29" t="s">
+        <v>459</v>
+      </c>
+      <c r="E198" s="40" t="s">
         <v>460</v>
-      </c>
-      <c r="E198" s="40" t="s">
-        <v>461</v>
       </c>
       <c r="F198" s="31"/>
       <c r="G198" s="31"/>
@@ -12307,13 +12310,13 @@
         <v>28</v>
       </c>
       <c r="C199" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D199" s="29" t="s">
+        <v>461</v>
+      </c>
+      <c r="E199" s="40" t="s">
         <v>462</v>
-      </c>
-      <c r="E199" s="40" t="s">
-        <v>463</v>
       </c>
       <c r="F199" s="31"/>
       <c r="G199" s="31"/>
@@ -12344,13 +12347,13 @@
         <v>28</v>
       </c>
       <c r="C200" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D200" s="29" t="s">
+        <v>463</v>
+      </c>
+      <c r="E200" s="40" t="s">
         <v>464</v>
-      </c>
-      <c r="E200" s="40" t="s">
-        <v>465</v>
       </c>
       <c r="F200" s="31"/>
       <c r="G200" s="31"/>
@@ -12381,13 +12384,13 @@
         <v>28</v>
       </c>
       <c r="C201" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D201" s="29" t="s">
+        <v>465</v>
+      </c>
+      <c r="E201" s="40" t="s">
         <v>466</v>
-      </c>
-      <c r="E201" s="40" t="s">
-        <v>467</v>
       </c>
       <c r="F201" s="31"/>
       <c r="G201" s="31"/>
@@ -12418,13 +12421,13 @@
         <v>28</v>
       </c>
       <c r="C202" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D202" s="29" t="s">
+        <v>467</v>
+      </c>
+      <c r="E202" s="40" t="s">
         <v>468</v>
-      </c>
-      <c r="E202" s="40" t="s">
-        <v>469</v>
       </c>
       <c r="F202" s="31"/>
       <c r="G202" s="31"/>
@@ -12455,13 +12458,13 @@
         <v>28</v>
       </c>
       <c r="C203" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D203" s="29" t="s">
+        <v>469</v>
+      </c>
+      <c r="E203" s="40" t="s">
         <v>470</v>
-      </c>
-      <c r="E203" s="40" t="s">
-        <v>471</v>
       </c>
       <c r="F203" s="31"/>
       <c r="G203" s="31"/>
@@ -12492,10 +12495,10 @@
         <v>28</v>
       </c>
       <c r="C204" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D204" s="29" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E204" s="37" t="s">
         <v>58</v>
@@ -12529,10 +12532,10 @@
         <v>28</v>
       </c>
       <c r="C205" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D205" s="29" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E205" s="37" t="s">
         <v>70</v>
@@ -12568,13 +12571,13 @@
         <v>28</v>
       </c>
       <c r="C206" s="35" t="s">
+        <v>473</v>
+      </c>
+      <c r="D206" s="29" t="s">
         <v>474</v>
       </c>
-      <c r="D206" s="29" t="s">
+      <c r="E206" s="40" t="s">
         <v>475</v>
-      </c>
-      <c r="E206" s="40" t="s">
-        <v>476</v>
       </c>
       <c r="F206" s="31"/>
       <c r="G206" s="31"/>
@@ -12605,13 +12608,13 @@
         <v>28</v>
       </c>
       <c r="C207" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D207" s="29" t="s">
+        <v>476</v>
+      </c>
+      <c r="E207" s="40" t="s">
         <v>477</v>
-      </c>
-      <c r="E207" s="40" t="s">
-        <v>478</v>
       </c>
       <c r="F207" s="31"/>
       <c r="G207" s="31"/>
@@ -12642,13 +12645,13 @@
         <v>28</v>
       </c>
       <c r="C208" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D208" s="29" t="s">
+        <v>478</v>
+      </c>
+      <c r="E208" s="40" t="s">
         <v>479</v>
-      </c>
-      <c r="E208" s="40" t="s">
-        <v>480</v>
       </c>
       <c r="F208" s="31"/>
       <c r="G208" s="31"/>
@@ -12679,13 +12682,13 @@
         <v>28</v>
       </c>
       <c r="C209" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D209" s="29" t="s">
+        <v>480</v>
+      </c>
+      <c r="E209" s="40" t="s">
         <v>481</v>
-      </c>
-      <c r="E209" s="40" t="s">
-        <v>482</v>
       </c>
       <c r="F209" s="31"/>
       <c r="G209" s="31"/>
@@ -12716,13 +12719,13 @@
         <v>28</v>
       </c>
       <c r="C210" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D210" s="29" t="s">
+        <v>482</v>
+      </c>
+      <c r="E210" s="40" t="s">
         <v>483</v>
-      </c>
-      <c r="E210" s="40" t="s">
-        <v>484</v>
       </c>
       <c r="F210" s="31"/>
       <c r="G210" s="31"/>
@@ -12753,13 +12756,13 @@
         <v>28</v>
       </c>
       <c r="C211" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D211" s="29" t="s">
+        <v>484</v>
+      </c>
+      <c r="E211" s="40" t="s">
         <v>485</v>
-      </c>
-      <c r="E211" s="40" t="s">
-        <v>486</v>
       </c>
       <c r="F211" s="31"/>
       <c r="G211" s="31"/>
@@ -12790,13 +12793,13 @@
         <v>28</v>
       </c>
       <c r="C212" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D212" s="29" t="s">
+        <v>486</v>
+      </c>
+      <c r="E212" s="40" t="s">
         <v>487</v>
-      </c>
-      <c r="E212" s="40" t="s">
-        <v>488</v>
       </c>
       <c r="F212" s="31"/>
       <c r="G212" s="31"/>
@@ -12827,13 +12830,13 @@
         <v>28</v>
       </c>
       <c r="C213" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D213" s="29" t="s">
+        <v>488</v>
+      </c>
+      <c r="E213" s="40" t="s">
         <v>489</v>
-      </c>
-      <c r="E213" s="40" t="s">
-        <v>490</v>
       </c>
       <c r="F213" s="31"/>
       <c r="G213" s="31"/>
@@ -12864,13 +12867,13 @@
         <v>28</v>
       </c>
       <c r="C214" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D214" s="29" t="s">
+        <v>490</v>
+      </c>
+      <c r="E214" s="40" t="s">
         <v>491</v>
-      </c>
-      <c r="E214" s="40" t="s">
-        <v>492</v>
       </c>
       <c r="F214" s="31"/>
       <c r="G214" s="31"/>
@@ -12901,13 +12904,13 @@
         <v>28</v>
       </c>
       <c r="C215" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D215" s="29" t="s">
+        <v>492</v>
+      </c>
+      <c r="E215" s="40" t="s">
         <v>493</v>
-      </c>
-      <c r="E215" s="40" t="s">
-        <v>494</v>
       </c>
       <c r="F215" s="31"/>
       <c r="G215" s="31"/>
@@ -12938,13 +12941,13 @@
         <v>28</v>
       </c>
       <c r="C216" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D216" s="29" t="s">
+        <v>494</v>
+      </c>
+      <c r="E216" s="40" t="s">
         <v>495</v>
-      </c>
-      <c r="E216" s="40" t="s">
-        <v>496</v>
       </c>
       <c r="F216" s="31"/>
       <c r="G216" s="31"/>
@@ -12975,13 +12978,13 @@
         <v>28</v>
       </c>
       <c r="C217" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D217" s="29" t="s">
+        <v>496</v>
+      </c>
+      <c r="E217" s="40" t="s">
         <v>497</v>
-      </c>
-      <c r="E217" s="40" t="s">
-        <v>498</v>
       </c>
       <c r="F217" s="31"/>
       <c r="G217" s="31"/>
@@ -13012,13 +13015,13 @@
         <v>28</v>
       </c>
       <c r="C218" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D218" s="29" t="s">
+        <v>498</v>
+      </c>
+      <c r="E218" s="40" t="s">
         <v>499</v>
-      </c>
-      <c r="E218" s="40" t="s">
-        <v>500</v>
       </c>
       <c r="F218" s="31"/>
       <c r="G218" s="31"/>
@@ -13049,10 +13052,10 @@
         <v>28</v>
       </c>
       <c r="C219" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D219" s="29" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="E219" s="37" t="s">
         <v>58</v>
@@ -13086,10 +13089,10 @@
         <v>28</v>
       </c>
       <c r="C220" s="35" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D220" s="29" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="E220" s="37" t="s">
         <v>70</v>
@@ -13125,13 +13128,13 @@
         <v>28</v>
       </c>
       <c r="C221" s="35" t="s">
+        <v>502</v>
+      </c>
+      <c r="D221" s="29" t="s">
         <v>503</v>
       </c>
-      <c r="D221" s="29" t="s">
+      <c r="E221" s="40" t="s">
         <v>504</v>
-      </c>
-      <c r="E221" s="40" t="s">
-        <v>505</v>
       </c>
       <c r="F221" s="31"/>
       <c r="G221" s="31"/>
@@ -13162,13 +13165,13 @@
         <v>28</v>
       </c>
       <c r="C222" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D222" s="29" t="s">
+        <v>505</v>
+      </c>
+      <c r="E222" s="40" t="s">
         <v>506</v>
-      </c>
-      <c r="E222" s="40" t="s">
-        <v>507</v>
       </c>
       <c r="F222" s="31"/>
       <c r="G222" s="31"/>
@@ -13199,13 +13202,13 @@
         <v>28</v>
       </c>
       <c r="C223" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D223" s="29" t="s">
+        <v>507</v>
+      </c>
+      <c r="E223" s="40" t="s">
         <v>508</v>
-      </c>
-      <c r="E223" s="40" t="s">
-        <v>509</v>
       </c>
       <c r="F223" s="31"/>
       <c r="G223" s="31"/>
@@ -13236,13 +13239,13 @@
         <v>28</v>
       </c>
       <c r="C224" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D224" s="29" t="s">
+        <v>509</v>
+      </c>
+      <c r="E224" s="40" t="s">
         <v>510</v>
-      </c>
-      <c r="E224" s="40" t="s">
-        <v>511</v>
       </c>
       <c r="F224" s="31"/>
       <c r="G224" s="31"/>
@@ -13273,13 +13276,13 @@
         <v>28</v>
       </c>
       <c r="C225" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D225" s="29" t="s">
+        <v>511</v>
+      </c>
+      <c r="E225" s="40" t="s">
         <v>512</v>
-      </c>
-      <c r="E225" s="40" t="s">
-        <v>513</v>
       </c>
       <c r="F225" s="31"/>
       <c r="G225" s="31"/>
@@ -13310,13 +13313,13 @@
         <v>28</v>
       </c>
       <c r="C226" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D226" s="29" t="s">
+        <v>513</v>
+      </c>
+      <c r="E226" s="40" t="s">
         <v>514</v>
-      </c>
-      <c r="E226" s="40" t="s">
-        <v>515</v>
       </c>
       <c r="F226" s="31"/>
       <c r="G226" s="31"/>
@@ -13347,13 +13350,13 @@
         <v>28</v>
       </c>
       <c r="C227" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D227" s="29" t="s">
+        <v>515</v>
+      </c>
+      <c r="E227" s="40" t="s">
         <v>516</v>
-      </c>
-      <c r="E227" s="40" t="s">
-        <v>517</v>
       </c>
       <c r="F227" s="31"/>
       <c r="G227" s="31"/>
@@ -13384,13 +13387,13 @@
         <v>28</v>
       </c>
       <c r="C228" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D228" s="29" t="s">
+        <v>517</v>
+      </c>
+      <c r="E228" s="40" t="s">
         <v>518</v>
-      </c>
-      <c r="E228" s="40" t="s">
-        <v>519</v>
       </c>
       <c r="F228" s="31"/>
       <c r="G228" s="31"/>
@@ -13421,13 +13424,13 @@
         <v>28</v>
       </c>
       <c r="C229" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D229" s="29" t="s">
+        <v>519</v>
+      </c>
+      <c r="E229" s="40" t="s">
         <v>520</v>
-      </c>
-      <c r="E229" s="40" t="s">
-        <v>521</v>
       </c>
       <c r="F229" s="31"/>
       <c r="G229" s="31"/>
@@ -13458,13 +13461,13 @@
         <v>28</v>
       </c>
       <c r="C230" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D230" s="29" t="s">
+        <v>521</v>
+      </c>
+      <c r="E230" s="40" t="s">
         <v>522</v>
-      </c>
-      <c r="E230" s="40" t="s">
-        <v>523</v>
       </c>
       <c r="F230" s="31"/>
       <c r="G230" s="31"/>
@@ -13495,13 +13498,13 @@
         <v>28</v>
       </c>
       <c r="C231" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D231" s="29" t="s">
+        <v>523</v>
+      </c>
+      <c r="E231" s="40" t="s">
         <v>524</v>
-      </c>
-      <c r="E231" s="40" t="s">
-        <v>525</v>
       </c>
       <c r="F231" s="31"/>
       <c r="G231" s="31"/>
@@ -13532,13 +13535,13 @@
         <v>28</v>
       </c>
       <c r="C232" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D232" s="29" t="s">
+        <v>525</v>
+      </c>
+      <c r="E232" s="40" t="s">
         <v>526</v>
-      </c>
-      <c r="E232" s="40" t="s">
-        <v>527</v>
       </c>
       <c r="F232" s="31"/>
       <c r="G232" s="31"/>
@@ -13569,13 +13572,13 @@
         <v>28</v>
       </c>
       <c r="C233" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D233" s="29" t="s">
+        <v>527</v>
+      </c>
+      <c r="E233" s="40" t="s">
         <v>528</v>
-      </c>
-      <c r="E233" s="40" t="s">
-        <v>529</v>
       </c>
       <c r="F233" s="31"/>
       <c r="G233" s="31"/>
@@ -13606,10 +13609,10 @@
         <v>28</v>
       </c>
       <c r="C234" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D234" s="29" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E234" s="37" t="s">
         <v>58</v>
@@ -13643,10 +13646,10 @@
         <v>28</v>
       </c>
       <c r="C235" s="35" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D235" s="29" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E235" s="37" t="s">
         <v>70</v>
@@ -13682,13 +13685,13 @@
         <v>28</v>
       </c>
       <c r="C236" s="42" t="s">
+        <v>531</v>
+      </c>
+      <c r="D236" s="41" t="s">
         <v>532</v>
       </c>
-      <c r="D236" s="41" t="s">
+      <c r="E236" s="40" t="s">
         <v>533</v>
-      </c>
-      <c r="E236" s="40" t="s">
-        <v>534</v>
       </c>
       <c r="F236" s="43"/>
       <c r="G236" s="43"/>
@@ -13719,13 +13722,13 @@
         <v>28</v>
       </c>
       <c r="C237" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D237" s="41" t="s">
+        <v>534</v>
+      </c>
+      <c r="E237" s="40" t="s">
         <v>535</v>
-      </c>
-      <c r="E237" s="40" t="s">
-        <v>536</v>
       </c>
       <c r="F237" s="43"/>
       <c r="G237" s="43"/>
@@ -13756,13 +13759,13 @@
         <v>28</v>
       </c>
       <c r="C238" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D238" s="41" t="s">
+        <v>536</v>
+      </c>
+      <c r="E238" s="40" t="s">
         <v>537</v>
-      </c>
-      <c r="E238" s="40" t="s">
-        <v>538</v>
       </c>
       <c r="F238" s="43"/>
       <c r="G238" s="43"/>
@@ -13793,13 +13796,13 @@
         <v>28</v>
       </c>
       <c r="C239" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D239" s="41" t="s">
+        <v>538</v>
+      </c>
+      <c r="E239" s="40" t="s">
         <v>539</v>
-      </c>
-      <c r="E239" s="40" t="s">
-        <v>540</v>
       </c>
       <c r="F239" s="43"/>
       <c r="G239" s="43"/>
@@ -13830,13 +13833,13 @@
         <v>28</v>
       </c>
       <c r="C240" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D240" s="41" t="s">
+        <v>540</v>
+      </c>
+      <c r="E240" s="40" t="s">
         <v>541</v>
-      </c>
-      <c r="E240" s="40" t="s">
-        <v>542</v>
       </c>
       <c r="F240" s="43"/>
       <c r="G240" s="43"/>
@@ -13867,13 +13870,13 @@
         <v>28</v>
       </c>
       <c r="C241" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D241" s="41" t="s">
+        <v>542</v>
+      </c>
+      <c r="E241" s="40" t="s">
         <v>543</v>
-      </c>
-      <c r="E241" s="40" t="s">
-        <v>544</v>
       </c>
       <c r="F241" s="43"/>
       <c r="G241" s="43"/>
@@ -13904,13 +13907,13 @@
         <v>28</v>
       </c>
       <c r="C242" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D242" s="41" t="s">
+        <v>544</v>
+      </c>
+      <c r="E242" s="40" t="s">
         <v>545</v>
-      </c>
-      <c r="E242" s="40" t="s">
-        <v>546</v>
       </c>
       <c r="F242" s="43"/>
       <c r="G242" s="43"/>
@@ -13941,13 +13944,13 @@
         <v>28</v>
       </c>
       <c r="C243" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D243" s="41" t="s">
+        <v>546</v>
+      </c>
+      <c r="E243" s="40" t="s">
         <v>547</v>
-      </c>
-      <c r="E243" s="40" t="s">
-        <v>548</v>
       </c>
       <c r="F243" s="43"/>
       <c r="G243" s="43"/>
@@ -13978,10 +13981,10 @@
         <v>28</v>
       </c>
       <c r="C244" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D244" s="41" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E244" s="40" t="s">
         <v>58</v>
@@ -14015,10 +14018,10 @@
         <v>28</v>
       </c>
       <c r="C245" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D245" s="41" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="E245" s="40" t="s">
         <v>70</v>
@@ -14054,13 +14057,13 @@
         <v>28</v>
       </c>
       <c r="C246" s="42" t="s">
+        <v>550</v>
+      </c>
+      <c r="D246" s="41" t="s">
         <v>551</v>
       </c>
-      <c r="D246" s="41" t="s">
+      <c r="E246" s="40" t="s">
         <v>552</v>
-      </c>
-      <c r="E246" s="40" t="s">
-        <v>553</v>
       </c>
       <c r="F246" s="43"/>
       <c r="G246" s="43"/>
@@ -14091,13 +14094,13 @@
         <v>28</v>
       </c>
       <c r="C247" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D247" s="41" t="s">
+        <v>553</v>
+      </c>
+      <c r="E247" s="40" t="s">
         <v>554</v>
-      </c>
-      <c r="E247" s="40" t="s">
-        <v>555</v>
       </c>
       <c r="F247" s="43"/>
       <c r="G247" s="43"/>
@@ -14128,13 +14131,13 @@
         <v>28</v>
       </c>
       <c r="C248" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D248" s="41" t="s">
+        <v>555</v>
+      </c>
+      <c r="E248" s="40" t="s">
         <v>556</v>
-      </c>
-      <c r="E248" s="40" t="s">
-        <v>557</v>
       </c>
       <c r="F248" s="43"/>
       <c r="G248" s="43"/>
@@ -14165,13 +14168,13 @@
         <v>28</v>
       </c>
       <c r="C249" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D249" s="41" t="s">
+        <v>557</v>
+      </c>
+      <c r="E249" s="40" t="s">
         <v>558</v>
-      </c>
-      <c r="E249" s="40" t="s">
-        <v>559</v>
       </c>
       <c r="F249" s="43"/>
       <c r="G249" s="43"/>
@@ -14202,13 +14205,13 @@
         <v>28</v>
       </c>
       <c r="C250" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D250" s="41" t="s">
+        <v>559</v>
+      </c>
+      <c r="E250" s="40" t="s">
         <v>560</v>
-      </c>
-      <c r="E250" s="40" t="s">
-        <v>561</v>
       </c>
       <c r="F250" s="43"/>
       <c r="G250" s="43"/>
@@ -14239,13 +14242,13 @@
         <v>28</v>
       </c>
       <c r="C251" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D251" s="41" t="s">
+        <v>561</v>
+      </c>
+      <c r="E251" s="40" t="s">
         <v>562</v>
-      </c>
-      <c r="E251" s="40" t="s">
-        <v>563</v>
       </c>
       <c r="F251" s="43"/>
       <c r="G251" s="43"/>
@@ -14276,13 +14279,13 @@
         <v>28</v>
       </c>
       <c r="C252" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D252" s="41" t="s">
+        <v>563</v>
+      </c>
+      <c r="E252" s="40" t="s">
         <v>564</v>
-      </c>
-      <c r="E252" s="40" t="s">
-        <v>565</v>
       </c>
       <c r="F252" s="43"/>
       <c r="G252" s="43"/>
@@ -14313,13 +14316,13 @@
         <v>28</v>
       </c>
       <c r="C253" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D253" s="41" t="s">
+        <v>565</v>
+      </c>
+      <c r="E253" s="40" t="s">
         <v>566</v>
-      </c>
-      <c r="E253" s="40" t="s">
-        <v>567</v>
       </c>
       <c r="F253" s="43"/>
       <c r="G253" s="43"/>
@@ -14350,13 +14353,13 @@
         <v>28</v>
       </c>
       <c r="C254" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D254" s="41" t="s">
+        <v>567</v>
+      </c>
+      <c r="E254" s="40" t="s">
         <v>568</v>
-      </c>
-      <c r="E254" s="40" t="s">
-        <v>569</v>
       </c>
       <c r="F254" s="43"/>
       <c r="G254" s="43"/>
@@ -14387,13 +14390,13 @@
         <v>28</v>
       </c>
       <c r="C255" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D255" s="41" t="s">
+        <v>569</v>
+      </c>
+      <c r="E255" s="40" t="s">
         <v>570</v>
-      </c>
-      <c r="E255" s="40" t="s">
-        <v>571</v>
       </c>
       <c r="F255" s="43"/>
       <c r="G255" s="43"/>
@@ -14424,13 +14427,13 @@
         <v>28</v>
       </c>
       <c r="C256" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D256" s="41" t="s">
+        <v>571</v>
+      </c>
+      <c r="E256" s="40" t="s">
         <v>572</v>
-      </c>
-      <c r="E256" s="40" t="s">
-        <v>573</v>
       </c>
       <c r="F256" s="43"/>
       <c r="G256" s="43"/>
@@ -14461,13 +14464,13 @@
         <v>28</v>
       </c>
       <c r="C257" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D257" s="41" t="s">
+        <v>573</v>
+      </c>
+      <c r="E257" s="40" t="s">
         <v>574</v>
-      </c>
-      <c r="E257" s="40" t="s">
-        <v>575</v>
       </c>
       <c r="F257" s="43"/>
       <c r="G257" s="43"/>
@@ -14498,13 +14501,13 @@
         <v>28</v>
       </c>
       <c r="C258" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D258" s="41" t="s">
+        <v>575</v>
+      </c>
+      <c r="E258" s="40" t="s">
         <v>576</v>
-      </c>
-      <c r="E258" s="40" t="s">
-        <v>577</v>
       </c>
       <c r="F258" s="43"/>
       <c r="G258" s="43"/>
@@ -14535,13 +14538,13 @@
         <v>28</v>
       </c>
       <c r="C259" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D259" s="41" t="s">
+        <v>577</v>
+      </c>
+      <c r="E259" s="40" t="s">
         <v>578</v>
-      </c>
-      <c r="E259" s="40" t="s">
-        <v>579</v>
       </c>
       <c r="F259" s="43"/>
       <c r="G259" s="43"/>
@@ -14572,13 +14575,13 @@
         <v>28</v>
       </c>
       <c r="C260" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D260" s="41" t="s">
+        <v>579</v>
+      </c>
+      <c r="E260" s="40" t="s">
         <v>580</v>
-      </c>
-      <c r="E260" s="40" t="s">
-        <v>581</v>
       </c>
       <c r="F260" s="43"/>
       <c r="G260" s="43"/>
@@ -14609,13 +14612,13 @@
         <v>28</v>
       </c>
       <c r="C261" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D261" s="41" t="s">
+        <v>581</v>
+      </c>
+      <c r="E261" s="40" t="s">
         <v>582</v>
-      </c>
-      <c r="E261" s="40" t="s">
-        <v>583</v>
       </c>
       <c r="F261" s="43"/>
       <c r="G261" s="43"/>
@@ -14646,13 +14649,13 @@
         <v>28</v>
       </c>
       <c r="C262" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D262" s="41" t="s">
+        <v>583</v>
+      </c>
+      <c r="E262" s="40" t="s">
         <v>584</v>
-      </c>
-      <c r="E262" s="40" t="s">
-        <v>585</v>
       </c>
       <c r="F262" s="43"/>
       <c r="G262" s="43"/>
@@ -14683,13 +14686,13 @@
         <v>28</v>
       </c>
       <c r="C263" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D263" s="41" t="s">
+        <v>585</v>
+      </c>
+      <c r="E263" s="40" t="s">
         <v>586</v>
-      </c>
-      <c r="E263" s="40" t="s">
-        <v>587</v>
       </c>
       <c r="F263" s="43"/>
       <c r="G263" s="43"/>
@@ -14720,10 +14723,10 @@
         <v>28</v>
       </c>
       <c r="C264" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D264" s="41" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="E264" s="40" t="s">
         <v>58</v>
@@ -14757,10 +14760,10 @@
         <v>28</v>
       </c>
       <c r="C265" s="42" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D265" s="41" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="E265" s="40" t="s">
         <v>70</v>
@@ -14796,13 +14799,13 @@
         <v>28</v>
       </c>
       <c r="C266" s="42" t="s">
+        <v>589</v>
+      </c>
+      <c r="D266" s="41" t="s">
         <v>590</v>
       </c>
-      <c r="D266" s="41" t="s">
+      <c r="E266" s="40" t="s">
         <v>591</v>
-      </c>
-      <c r="E266" s="40" t="s">
-        <v>592</v>
       </c>
       <c r="F266" s="43"/>
       <c r="G266" s="43"/>
@@ -14833,13 +14836,13 @@
         <v>28</v>
       </c>
       <c r="C267" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D267" s="41" t="s">
+        <v>592</v>
+      </c>
+      <c r="E267" s="40" t="s">
         <v>593</v>
-      </c>
-      <c r="E267" s="40" t="s">
-        <v>594</v>
       </c>
       <c r="F267" s="43"/>
       <c r="G267" s="43"/>
@@ -14870,13 +14873,13 @@
         <v>28</v>
       </c>
       <c r="C268" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D268" s="41" t="s">
+        <v>594</v>
+      </c>
+      <c r="E268" s="40" t="s">
         <v>595</v>
-      </c>
-      <c r="E268" s="40" t="s">
-        <v>596</v>
       </c>
       <c r="F268" s="43"/>
       <c r="G268" s="43"/>
@@ -14907,13 +14910,13 @@
         <v>28</v>
       </c>
       <c r="C269" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D269" s="41" t="s">
+        <v>596</v>
+      </c>
+      <c r="E269" s="40" t="s">
         <v>597</v>
-      </c>
-      <c r="E269" s="40" t="s">
-        <v>598</v>
       </c>
       <c r="F269" s="43"/>
       <c r="G269" s="43"/>
@@ -14944,13 +14947,13 @@
         <v>28</v>
       </c>
       <c r="C270" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D270" s="41" t="s">
+        <v>598</v>
+      </c>
+      <c r="E270" s="40" t="s">
         <v>599</v>
-      </c>
-      <c r="E270" s="40" t="s">
-        <v>600</v>
       </c>
       <c r="F270" s="43"/>
       <c r="G270" s="43"/>
@@ -14981,13 +14984,13 @@
         <v>28</v>
       </c>
       <c r="C271" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D271" s="41" t="s">
+        <v>600</v>
+      </c>
+      <c r="E271" s="40" t="s">
         <v>601</v>
-      </c>
-      <c r="E271" s="40" t="s">
-        <v>602</v>
       </c>
       <c r="F271" s="43"/>
       <c r="G271" s="43"/>
@@ -15018,13 +15021,13 @@
         <v>28</v>
       </c>
       <c r="C272" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D272" s="41" t="s">
+        <v>602</v>
+      </c>
+      <c r="E272" s="40" t="s">
         <v>603</v>
-      </c>
-      <c r="E272" s="40" t="s">
-        <v>604</v>
       </c>
       <c r="F272" s="43"/>
       <c r="G272" s="43"/>
@@ -15055,13 +15058,13 @@
         <v>28</v>
       </c>
       <c r="C273" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D273" s="41" t="s">
+        <v>604</v>
+      </c>
+      <c r="E273" s="40" t="s">
         <v>605</v>
-      </c>
-      <c r="E273" s="40" t="s">
-        <v>606</v>
       </c>
       <c r="F273" s="43"/>
       <c r="G273" s="43"/>
@@ -15092,13 +15095,13 @@
         <v>28</v>
       </c>
       <c r="C274" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D274" s="41" t="s">
+        <v>606</v>
+      </c>
+      <c r="E274" s="40" t="s">
         <v>607</v>
-      </c>
-      <c r="E274" s="40" t="s">
-        <v>608</v>
       </c>
       <c r="F274" s="43"/>
       <c r="G274" s="43"/>
@@ -15129,13 +15132,13 @@
         <v>28</v>
       </c>
       <c r="C275" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D275" s="41" t="s">
+        <v>608</v>
+      </c>
+      <c r="E275" s="40" t="s">
         <v>609</v>
-      </c>
-      <c r="E275" s="40" t="s">
-        <v>610</v>
       </c>
       <c r="F275" s="43"/>
       <c r="G275" s="43"/>
@@ -15166,13 +15169,13 @@
         <v>28</v>
       </c>
       <c r="C276" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D276" s="41" t="s">
+        <v>610</v>
+      </c>
+      <c r="E276" s="40" t="s">
         <v>611</v>
-      </c>
-      <c r="E276" s="40" t="s">
-        <v>612</v>
       </c>
       <c r="F276" s="43"/>
       <c r="G276" s="43"/>
@@ -15203,13 +15206,13 @@
         <v>28</v>
       </c>
       <c r="C277" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D277" s="41" t="s">
+        <v>612</v>
+      </c>
+      <c r="E277" s="40" t="s">
         <v>613</v>
-      </c>
-      <c r="E277" s="40" t="s">
-        <v>614</v>
       </c>
       <c r="F277" s="43"/>
       <c r="G277" s="43"/>
@@ -15240,13 +15243,13 @@
         <v>28</v>
       </c>
       <c r="C278" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D278" s="41" t="s">
+        <v>614</v>
+      </c>
+      <c r="E278" s="40" t="s">
         <v>615</v>
-      </c>
-      <c r="E278" s="40" t="s">
-        <v>616</v>
       </c>
       <c r="F278" s="43"/>
       <c r="G278" s="43"/>
@@ -15277,13 +15280,13 @@
         <v>28</v>
       </c>
       <c r="C279" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D279" s="41" t="s">
+        <v>616</v>
+      </c>
+      <c r="E279" s="40" t="s">
         <v>617</v>
-      </c>
-      <c r="E279" s="40" t="s">
-        <v>618</v>
       </c>
       <c r="F279" s="43"/>
       <c r="G279" s="43"/>
@@ -15314,13 +15317,13 @@
         <v>28</v>
       </c>
       <c r="C280" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D280" s="41" t="s">
+        <v>618</v>
+      </c>
+      <c r="E280" s="40" t="s">
         <v>619</v>
-      </c>
-      <c r="E280" s="40" t="s">
-        <v>620</v>
       </c>
       <c r="F280" s="43"/>
       <c r="G280" s="43"/>
@@ -15351,13 +15354,13 @@
         <v>28</v>
       </c>
       <c r="C281" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D281" s="41" t="s">
+        <v>620</v>
+      </c>
+      <c r="E281" s="40" t="s">
         <v>621</v>
-      </c>
-      <c r="E281" s="40" t="s">
-        <v>622</v>
       </c>
       <c r="F281" s="43"/>
       <c r="G281" s="43"/>
@@ -15388,13 +15391,13 @@
         <v>28</v>
       </c>
       <c r="C282" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D282" s="41" t="s">
+        <v>622</v>
+      </c>
+      <c r="E282" s="40" t="s">
         <v>623</v>
-      </c>
-      <c r="E282" s="40" t="s">
-        <v>624</v>
       </c>
       <c r="F282" s="43"/>
       <c r="G282" s="43"/>
@@ -15425,13 +15428,13 @@
         <v>28</v>
       </c>
       <c r="C283" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D283" s="41" t="s">
+        <v>624</v>
+      </c>
+      <c r="E283" s="40" t="s">
         <v>625</v>
-      </c>
-      <c r="E283" s="40" t="s">
-        <v>626</v>
       </c>
       <c r="F283" s="43"/>
       <c r="G283" s="43"/>
@@ -15462,10 +15465,10 @@
         <v>28</v>
       </c>
       <c r="C284" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D284" s="41" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="E284" s="40" t="s">
         <v>58</v>
@@ -15499,10 +15502,10 @@
         <v>28</v>
       </c>
       <c r="C285" s="42" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D285" s="41" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="E285" s="40" t="s">
         <v>70</v>
@@ -15540,7 +15543,7 @@
       <c r="L286" s="7"/>
       <c r="M286" s="7"/>
       <c r="N286" s="7"/>
-      <c r="O286" s="72"/>
+      <c r="O286" s="60"/>
       <c r="P286" s="7"/>
       <c r="Q286" s="7"/>
       <c r="R286" s="7"/>
@@ -15560,7 +15563,7 @@
       <c r="L287" s="7"/>
       <c r="M287" s="7"/>
       <c r="N287" s="7"/>
-      <c r="O287" s="72"/>
+      <c r="O287" s="60"/>
       <c r="P287" s="7"/>
       <c r="Q287" s="7"/>
       <c r="R287" s="7"/>
@@ -15580,7 +15583,7 @@
       <c r="L288" s="7"/>
       <c r="M288" s="7"/>
       <c r="N288" s="7"/>
-      <c r="O288" s="72"/>
+      <c r="O288" s="60"/>
       <c r="P288" s="7"/>
       <c r="Q288" s="7"/>
       <c r="R288" s="7"/>
@@ -15600,7 +15603,7 @@
       <c r="L289" s="7"/>
       <c r="M289" s="7"/>
       <c r="N289" s="7"/>
-      <c r="O289" s="72"/>
+      <c r="O289" s="60"/>
       <c r="P289" s="7"/>
       <c r="Q289" s="7"/>
       <c r="R289" s="7"/>
@@ -15620,7 +15623,7 @@
       <c r="L290" s="7"/>
       <c r="M290" s="7"/>
       <c r="N290" s="7"/>
-      <c r="O290" s="72"/>
+      <c r="O290" s="60"/>
       <c r="P290" s="7"/>
       <c r="Q290" s="7"/>
       <c r="R290" s="7"/>
@@ -15640,7 +15643,7 @@
       <c r="L291" s="7"/>
       <c r="M291" s="7"/>
       <c r="N291" s="7"/>
-      <c r="O291" s="72"/>
+      <c r="O291" s="60"/>
       <c r="P291" s="7"/>
       <c r="Q291" s="7"/>
       <c r="R291" s="7"/>
@@ -15660,7 +15663,7 @@
       <c r="L292" s="7"/>
       <c r="M292" s="7"/>
       <c r="N292" s="7"/>
-      <c r="O292" s="72"/>
+      <c r="O292" s="60"/>
       <c r="P292" s="7"/>
       <c r="Q292" s="7"/>
       <c r="R292" s="7"/>
@@ -15680,7 +15683,7 @@
       <c r="L293" s="7"/>
       <c r="M293" s="7"/>
       <c r="N293" s="7"/>
-      <c r="O293" s="72"/>
+      <c r="O293" s="60"/>
       <c r="P293" s="7"/>
       <c r="Q293" s="7"/>
       <c r="R293" s="7"/>
@@ -15700,7 +15703,7 @@
       <c r="L294" s="7"/>
       <c r="M294" s="7"/>
       <c r="N294" s="7"/>
-      <c r="O294" s="72"/>
+      <c r="O294" s="60"/>
       <c r="P294" s="7"/>
       <c r="Q294" s="7"/>
       <c r="R294" s="7"/>
@@ -15720,7 +15723,7 @@
       <c r="L295" s="7"/>
       <c r="M295" s="7"/>
       <c r="N295" s="7"/>
-      <c r="O295" s="72"/>
+      <c r="O295" s="60"/>
       <c r="P295" s="7"/>
       <c r="Q295" s="7"/>
       <c r="R295" s="7"/>
@@ -15740,7 +15743,7 @@
       <c r="L296" s="7"/>
       <c r="M296" s="7"/>
       <c r="N296" s="7"/>
-      <c r="O296" s="72"/>
+      <c r="O296" s="60"/>
       <c r="P296" s="7"/>
       <c r="Q296" s="7"/>
       <c r="R296" s="7"/>
@@ -15760,7 +15763,7 @@
       <c r="L297" s="7"/>
       <c r="M297" s="7"/>
       <c r="N297" s="7"/>
-      <c r="O297" s="72"/>
+      <c r="O297" s="60"/>
       <c r="P297" s="7"/>
       <c r="Q297" s="7"/>
       <c r="R297" s="7"/>
@@ -15780,7 +15783,7 @@
       <c r="L298" s="7"/>
       <c r="M298" s="7"/>
       <c r="N298" s="7"/>
-      <c r="O298" s="72"/>
+      <c r="O298" s="60"/>
       <c r="P298" s="7"/>
       <c r="Q298" s="7"/>
       <c r="R298" s="7"/>
@@ -15800,7 +15803,7 @@
       <c r="L299" s="7"/>
       <c r="M299" s="7"/>
       <c r="N299" s="7"/>
-      <c r="O299" s="72"/>
+      <c r="O299" s="60"/>
       <c r="P299" s="7"/>
       <c r="Q299" s="7"/>
       <c r="R299" s="7"/>
@@ -15820,7 +15823,7 @@
       <c r="L300" s="7"/>
       <c r="M300" s="7"/>
       <c r="N300" s="7"/>
-      <c r="O300" s="72"/>
+      <c r="O300" s="60"/>
       <c r="P300" s="7"/>
       <c r="Q300" s="7"/>
       <c r="R300" s="7"/>
@@ -15840,7 +15843,7 @@
       <c r="L301" s="7"/>
       <c r="M301" s="7"/>
       <c r="N301" s="7"/>
-      <c r="O301" s="72"/>
+      <c r="O301" s="60"/>
       <c r="P301" s="7"/>
       <c r="Q301" s="7"/>
       <c r="R301" s="7"/>
@@ -15860,7 +15863,7 @@
       <c r="L302" s="7"/>
       <c r="M302" s="7"/>
       <c r="N302" s="7"/>
-      <c r="O302" s="72"/>
+      <c r="O302" s="60"/>
       <c r="P302" s="7"/>
       <c r="Q302" s="7"/>
       <c r="R302" s="7"/>
@@ -15880,7 +15883,7 @@
       <c r="L303" s="7"/>
       <c r="M303" s="7"/>
       <c r="N303" s="7"/>
-      <c r="O303" s="72"/>
+      <c r="O303" s="60"/>
       <c r="P303" s="7"/>
       <c r="Q303" s="7"/>
       <c r="R303" s="7"/>
@@ -15900,7 +15903,7 @@
       <c r="L304" s="7"/>
       <c r="M304" s="7"/>
       <c r="N304" s="7"/>
-      <c r="O304" s="72"/>
+      <c r="O304" s="60"/>
       <c r="P304" s="7"/>
       <c r="Q304" s="7"/>
       <c r="R304" s="7"/>
@@ -15920,7 +15923,7 @@
       <c r="L305" s="7"/>
       <c r="M305" s="7"/>
       <c r="N305" s="7"/>
-      <c r="O305" s="72"/>
+      <c r="O305" s="60"/>
       <c r="P305" s="7"/>
       <c r="Q305" s="7"/>
       <c r="R305" s="7"/>
@@ -15940,7 +15943,7 @@
       <c r="L306" s="7"/>
       <c r="M306" s="7"/>
       <c r="N306" s="7"/>
-      <c r="O306" s="72"/>
+      <c r="O306" s="60"/>
       <c r="P306" s="7"/>
       <c r="Q306" s="7"/>
       <c r="R306" s="7"/>
@@ -15960,7 +15963,7 @@
       <c r="L307" s="7"/>
       <c r="M307" s="7"/>
       <c r="N307" s="7"/>
-      <c r="O307" s="72"/>
+      <c r="O307" s="60"/>
       <c r="P307" s="7"/>
       <c r="Q307" s="7"/>
       <c r="R307" s="7"/>
@@ -15980,7 +15983,7 @@
       <c r="L308" s="7"/>
       <c r="M308" s="7"/>
       <c r="N308" s="7"/>
-      <c r="O308" s="72"/>
+      <c r="O308" s="60"/>
       <c r="P308" s="7"/>
       <c r="Q308" s="7"/>
       <c r="R308" s="7"/>
@@ -16000,7 +16003,7 @@
       <c r="L309" s="7"/>
       <c r="M309" s="7"/>
       <c r="N309" s="7"/>
-      <c r="O309" s="72"/>
+      <c r="O309" s="60"/>
       <c r="P309" s="7"/>
       <c r="Q309" s="7"/>
       <c r="R309" s="7"/>
@@ -16020,7 +16023,7 @@
       <c r="L310" s="7"/>
       <c r="M310" s="7"/>
       <c r="N310" s="7"/>
-      <c r="O310" s="72"/>
+      <c r="O310" s="60"/>
       <c r="P310" s="7"/>
       <c r="Q310" s="7"/>
       <c r="R310" s="7"/>
@@ -16040,7 +16043,7 @@
       <c r="L311" s="7"/>
       <c r="M311" s="7"/>
       <c r="N311" s="7"/>
-      <c r="O311" s="72"/>
+      <c r="O311" s="60"/>
       <c r="P311" s="7"/>
       <c r="Q311" s="7"/>
       <c r="R311" s="7"/>
@@ -16060,7 +16063,7 @@
       <c r="L312" s="7"/>
       <c r="M312" s="7"/>
       <c r="N312" s="7"/>
-      <c r="O312" s="72"/>
+      <c r="O312" s="60"/>
       <c r="P312" s="7"/>
       <c r="Q312" s="7"/>
       <c r="R312" s="7"/>
@@ -16080,7 +16083,7 @@
       <c r="L313" s="7"/>
       <c r="M313" s="7"/>
       <c r="N313" s="7"/>
-      <c r="O313" s="72"/>
+      <c r="O313" s="60"/>
       <c r="P313" s="7"/>
       <c r="Q313" s="7"/>
       <c r="R313" s="7"/>
@@ -16100,7 +16103,7 @@
       <c r="L314" s="7"/>
       <c r="M314" s="7"/>
       <c r="N314" s="7"/>
-      <c r="O314" s="72"/>
+      <c r="O314" s="60"/>
       <c r="P314" s="7"/>
       <c r="Q314" s="7"/>
       <c r="R314" s="7"/>
@@ -16120,7 +16123,7 @@
       <c r="L315" s="7"/>
       <c r="M315" s="7"/>
       <c r="N315" s="7"/>
-      <c r="O315" s="72"/>
+      <c r="O315" s="60"/>
       <c r="P315" s="7"/>
       <c r="Q315" s="7"/>
       <c r="R315" s="7"/>
@@ -16140,7 +16143,7 @@
       <c r="L316" s="7"/>
       <c r="M316" s="7"/>
       <c r="N316" s="7"/>
-      <c r="O316" s="72"/>
+      <c r="O316" s="60"/>
       <c r="P316" s="7"/>
       <c r="Q316" s="7"/>
       <c r="R316" s="7"/>
@@ -16160,7 +16163,7 @@
       <c r="L317" s="7"/>
       <c r="M317" s="7"/>
       <c r="N317" s="7"/>
-      <c r="O317" s="72"/>
+      <c r="O317" s="60"/>
       <c r="P317" s="7"/>
       <c r="Q317" s="7"/>
       <c r="R317" s="7"/>
@@ -16180,7 +16183,7 @@
       <c r="L318" s="7"/>
       <c r="M318" s="7"/>
       <c r="N318" s="7"/>
-      <c r="O318" s="72"/>
+      <c r="O318" s="60"/>
       <c r="P318" s="7"/>
       <c r="Q318" s="7"/>
       <c r="R318" s="7"/>
@@ -16200,7 +16203,7 @@
       <c r="L319" s="7"/>
       <c r="M319" s="7"/>
       <c r="N319" s="7"/>
-      <c r="O319" s="72"/>
+      <c r="O319" s="60"/>
       <c r="P319" s="7"/>
       <c r="Q319" s="7"/>
       <c r="R319" s="7"/>
@@ -16220,7 +16223,7 @@
       <c r="L320" s="7"/>
       <c r="M320" s="7"/>
       <c r="N320" s="7"/>
-      <c r="O320" s="72"/>
+      <c r="O320" s="60"/>
       <c r="P320" s="7"/>
       <c r="Q320" s="7"/>
       <c r="R320" s="7"/>
@@ -16240,7 +16243,7 @@
       <c r="L321" s="7"/>
       <c r="M321" s="7"/>
       <c r="N321" s="7"/>
-      <c r="O321" s="72"/>
+      <c r="O321" s="60"/>
       <c r="P321" s="7"/>
       <c r="Q321" s="7"/>
       <c r="R321" s="7"/>
@@ -16260,7 +16263,7 @@
       <c r="L322" s="7"/>
       <c r="M322" s="7"/>
       <c r="N322" s="7"/>
-      <c r="O322" s="72"/>
+      <c r="O322" s="60"/>
       <c r="P322" s="7"/>
       <c r="Q322" s="7"/>
       <c r="R322" s="7"/>
@@ -16280,7 +16283,7 @@
       <c r="L323" s="7"/>
       <c r="M323" s="7"/>
       <c r="N323" s="7"/>
-      <c r="O323" s="72"/>
+      <c r="O323" s="60"/>
       <c r="P323" s="7"/>
       <c r="Q323" s="7"/>
       <c r="R323" s="7"/>
@@ -16300,7 +16303,7 @@
       <c r="L324" s="7"/>
       <c r="M324" s="7"/>
       <c r="N324" s="7"/>
-      <c r="O324" s="72"/>
+      <c r="O324" s="60"/>
       <c r="P324" s="7"/>
       <c r="Q324" s="7"/>
       <c r="R324" s="7"/>
@@ -16320,7 +16323,7 @@
       <c r="L325" s="7"/>
       <c r="M325" s="7"/>
       <c r="N325" s="7"/>
-      <c r="O325" s="72"/>
+      <c r="O325" s="60"/>
       <c r="P325" s="7"/>
       <c r="Q325" s="7"/>
       <c r="R325" s="7"/>
@@ -16340,7 +16343,7 @@
       <c r="L326" s="7"/>
       <c r="M326" s="7"/>
       <c r="N326" s="7"/>
-      <c r="O326" s="72"/>
+      <c r="O326" s="60"/>
       <c r="P326" s="7"/>
       <c r="Q326" s="7"/>
       <c r="R326" s="7"/>
@@ -16360,7 +16363,7 @@
       <c r="L327" s="7"/>
       <c r="M327" s="7"/>
       <c r="N327" s="7"/>
-      <c r="O327" s="72"/>
+      <c r="O327" s="60"/>
       <c r="P327" s="7"/>
       <c r="Q327" s="7"/>
       <c r="R327" s="7"/>
@@ -16380,7 +16383,7 @@
       <c r="L328" s="7"/>
       <c r="M328" s="7"/>
       <c r="N328" s="7"/>
-      <c r="O328" s="72"/>
+      <c r="O328" s="60"/>
       <c r="P328" s="7"/>
       <c r="Q328" s="7"/>
       <c r="R328" s="7"/>
@@ -16400,7 +16403,7 @@
       <c r="L329" s="7"/>
       <c r="M329" s="7"/>
       <c r="N329" s="7"/>
-      <c r="O329" s="72"/>
+      <c r="O329" s="60"/>
       <c r="P329" s="7"/>
       <c r="Q329" s="7"/>
       <c r="R329" s="7"/>
@@ -16420,7 +16423,7 @@
       <c r="L330" s="7"/>
       <c r="M330" s="7"/>
       <c r="N330" s="7"/>
-      <c r="O330" s="72"/>
+      <c r="O330" s="60"/>
       <c r="P330" s="7"/>
       <c r="Q330" s="7"/>
       <c r="R330" s="7"/>
@@ -16440,7 +16443,7 @@
       <c r="L331" s="7"/>
       <c r="M331" s="7"/>
       <c r="N331" s="7"/>
-      <c r="O331" s="72"/>
+      <c r="O331" s="60"/>
       <c r="P331" s="7"/>
       <c r="Q331" s="7"/>
       <c r="R331" s="7"/>
@@ -17736,42 +17739,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
   </sheetData>
@@ -17795,22 +17798,22 @@
   <sheetData>
     <row r="1" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="11" t="s">
+        <v>655</v>
+      </c>
+      <c r="D1" s="51" t="s">
         <v>656</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="F1" s="12" t="s">
         <v>657</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="39" t="s">
         <v>658</v>
-      </c>
-      <c r="G1" s="39" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -17818,13 +17821,13 @@
         <v>29</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="C2" s="49" t="s">
         <v>660</v>
       </c>
-      <c r="C2" s="49" t="s">
+      <c r="D2" s="52" t="s">
         <v>661</v>
-      </c>
-      <c r="D2" s="52" t="s">
-        <v>662</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -17832,13 +17835,13 @@
         <v>36</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C3" s="49" t="s">
+        <v>662</v>
+      </c>
+      <c r="D3" s="53" t="s">
         <v>663</v>
-      </c>
-      <c r="D3" s="53" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -17846,13 +17849,13 @@
         <v>47</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C4" s="49" t="s">
+        <v>664</v>
+      </c>
+      <c r="D4" s="54" t="s">
         <v>665</v>
-      </c>
-      <c r="D4" s="54" t="s">
-        <v>666</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -17860,13 +17863,13 @@
         <v>51</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C5" s="49" t="s">
+        <v>666</v>
+      </c>
+      <c r="D5" s="53" t="s">
         <v>667</v>
-      </c>
-      <c r="D5" s="53" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -17874,13 +17877,13 @@
         <v>53</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C6" s="49" t="s">
+        <v>668</v>
+      </c>
+      <c r="D6" s="54" t="s">
         <v>669</v>
-      </c>
-      <c r="D6" s="54" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -17888,13 +17891,13 @@
         <v>55</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C7" s="49" t="s">
+        <v>670</v>
+      </c>
+      <c r="D7" s="54" t="s">
         <v>671</v>
-      </c>
-      <c r="D7" s="54" t="s">
-        <v>672</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -17902,13 +17905,13 @@
         <v>49</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C8" s="49" t="s">
+        <v>672</v>
+      </c>
+      <c r="D8" s="54" t="s">
         <v>673</v>
-      </c>
-      <c r="D8" s="54" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -17916,27 +17919,27 @@
         <v>45</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C9" s="49" t="s">
+        <v>674</v>
+      </c>
+      <c r="D9" s="54" t="s">
         <v>675</v>
-      </c>
-      <c r="D9" s="54" t="s">
-        <v>676</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="C10" s="50" t="s">
         <v>677</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="C10" s="50" t="s">
+      <c r="D10" s="53" t="s">
         <v>678</v>
-      </c>
-      <c r="D10" s="53" t="s">
-        <v>679</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -17944,97 +17947,97 @@
         <v>347</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C11" s="49" t="s">
+        <v>679</v>
+      </c>
+      <c r="D11" s="54" t="s">
         <v>680</v>
-      </c>
-      <c r="D11" s="54" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C12" s="49" t="s">
+        <v>681</v>
+      </c>
+      <c r="D12" s="54" t="s">
         <v>682</v>
-      </c>
-      <c r="D12" s="54" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C13" s="49" t="s">
+        <v>683</v>
+      </c>
+      <c r="D13" s="54" t="s">
         <v>684</v>
-      </c>
-      <c r="D13" s="54" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C14" s="49" t="s">
+        <v>685</v>
+      </c>
+      <c r="D14" s="54" t="s">
         <v>686</v>
-      </c>
-      <c r="D14" s="54" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C15" s="49">
         <v>521</v>
       </c>
       <c r="D15" s="54" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="56" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C16" s="58" t="s">
+        <v>688</v>
+      </c>
+      <c r="D16" s="54" t="s">
         <v>689</v>
-      </c>
-      <c r="D16" s="54" t="s">
-        <v>690</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="57" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B17" s="55" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C17" s="59" t="s">
+        <v>690</v>
+      </c>
+      <c r="D17" s="54" t="s">
         <v>691</v>
-      </c>
-      <c r="D17" s="54" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -19015,7 +19018,7 @@
     </row>
     <row r="3" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>73</v>

</xml_diff>